<commit_message>
feat: Implement banner carousel and update costume card functionality
- Added a new banner image (banner-4.jpg) and implemented an automatic rotation for the hero banner images.
- Enhanced the costume card rendering to support grouping by variants, allowing navigation between different costume variants.
- Updated the modal functionality to display costume variants with navigation arrows.
- Improved search functionality to include keywords for filtering costumes.
- Refactored popular costumes logic to randomly select one costume from each gender category instead of relying on click counts.
- Updated translations and category options in the filters.
- Added error handling for images and improved the loading experience.
</commit_message>
<xml_diff>
--- a/inventario-disfraces.xlsx
+++ b/inventario-disfraces.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -463,6 +463,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,6 +502,11 @@
           <t>Palabras Clave</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Grupo de Diseño</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -536,6 +542,11 @@
           <t>bombero, fireman, extintor, incendio, rescate, uniforme, profesion, disfraz escolar</t>
         </is>
       </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>bombero</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -571,6 +582,11 @@
           <t>charro, mexico, mexicano, sombrero, folclorico, tradicional, dia de muertos, fiestas patrias</t>
         </is>
       </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>charro-mexicano</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -606,6 +622,11 @@
           <t>detective, sherlock, investigador, gabardina, lupa, misterio, disfraz de epoca</t>
         </is>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>detective</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -641,6 +662,11 @@
           <t>espantapajaros, scarecrow, halloween, paja, granja, mago de oz</t>
         </is>
       </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>espantapajaros</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -676,6 +702,11 @@
           <t>gaucho, argentina, poncho, folclorico, tradicional, campo</t>
         </is>
       </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>gaucho</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -711,6 +742,11 @@
           <t>hombre lobo, lobo, werewolf, halloween, monstruo, licantropo</t>
         </is>
       </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>hombre-lobo</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -746,6 +782,11 @@
           <t>san jose, jose, biblico, nacimiento, pesebre, pase del nino, navidad religiosa</t>
         </is>
       </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>san-jose</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -781,6 +822,11 @@
           <t>kimono, japon, japones, oriental, tradicional, asiatico</t>
         </is>
       </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>kimono</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -816,6 +862,11 @@
           <t>marinero, sailor, nautico, barco, capitan, mar</t>
         </is>
       </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>marinero</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -851,6 +902,11 @@
           <t>caballero, medieval, armadura, gladiador, espada, edad media, epoca</t>
         </is>
       </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>medieval-caballero</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -886,6 +942,11 @@
           <t>montubio, costa, ecuador, folclorico, tradicional, campesino</t>
         </is>
       </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>montubio</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -921,6 +982,11 @@
           <t>papa noel, santa claus, navidad, santa, gorro rojo</t>
         </is>
       </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>papa-noel</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -956,6 +1022,11 @@
           <t>payaso siniestro, clown, payaso malo, halloween, terror, miedo</t>
         </is>
       </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>payaso-siniestro</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -991,6 +1062,11 @@
           <t>piloto, aviador, avion, uniforme, profesion, capitan</t>
         </is>
       </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>piloto</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1026,6 +1102,11 @@
           <t>rey mago, reyes magos, melchor, gaspar, baltazar, pesebre, pase del nino</t>
         </is>
       </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>rey-mago</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1061,6 +1142,11 @@
           <t>romano, roma, gladiador, epoca, historico, imperio romano</t>
         </is>
       </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>romano</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1096,6 +1182,11 @@
           <t>vampiro, dracula, halloween, capa, colmillos, gotico</t>
         </is>
       </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>vampiro-clasico</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1131,6 +1222,11 @@
           <t>vaquero, cowboy, oeste, western, sombrero, rancho</t>
         </is>
       </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>vaquero-oeste</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1166,6 +1262,11 @@
           <t>vikingo, viking, nordico, casco cuernos, guerrero, epoca</t>
         </is>
       </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>vikingo</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1201,6 +1302,11 @@
           <t>astronauta, espacio, nasa, cosmonauta, profesion</t>
         </is>
       </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>astronauta</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1236,6 +1342,11 @@
           <t>bruja, hechicera, halloween, magia, sombrero puntiagudo, escoba</t>
         </is>
       </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>bruja</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1271,6 +1382,11 @@
           <t>catrina, dia de muertos, mexico, calavera, mexicano, halloween mexicano</t>
         </is>
       </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>catrina</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1306,6 +1422,11 @@
           <t>chola cuencana, chola, cuenca, folclorico, ecuador, pollera, traje tipico</t>
         </is>
       </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>chola-cuencana</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1341,6 +1462,11 @@
           <t>cientifica, laboratorio, quimica, profesion, bata blanca</t>
         </is>
       </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>cientifico</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1376,6 +1502,11 @@
           <t>diabla, diablo, halloween, cuernos, tridente, rojo</t>
         </is>
       </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>diablo</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1411,6 +1542,11 @@
           <t>egipcia, egipto, faraon, cleopatra, epoca, antiguo egipto</t>
         </is>
       </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>egipcio</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1446,6 +1582,11 @@
           <t>esqueleto, huesos, halloween, calavera, dia de muertos</t>
         </is>
       </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>esqueleto</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1481,6 +1622,11 @@
           <t>fantasma, ghost, halloween, sabana, espiritu</t>
         </is>
       </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>fantasma</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1516,6 +1662,11 @@
           <t>flamenca, espana, espanol, lunares, baile, folclorico</t>
         </is>
       </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>flamenca</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1551,6 +1702,11 @@
           <t>granjera, campo, agricultora, profesion, overol</t>
         </is>
       </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>granjero</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1586,6 +1742,11 @@
           <t>griega, grecia, diosa griega, toga, epoca, antigua grecia</t>
         </is>
       </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>griego</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1621,6 +1782,11 @@
           <t>hawaiana, hawaii, tropical, playa, collar flores, verano</t>
         </is>
       </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>hawaiano</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1656,6 +1822,11 @@
           <t>virgen maria, maria, biblico, nacimiento, pesebre, pase del nino</t>
         </is>
       </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>virgen-maria</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1691,6 +1862,11 @@
           <t>doctora, medica, medico, profesion, bata blanca, estetoscopio</t>
         </is>
       </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>doctor</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1726,6 +1902,11 @@
           <t>dama medieval, medieval, princesa medieval, epoca, edad media</t>
         </is>
       </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>medieval-dama</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1761,6 +1942,11 @@
           <t>momia, egipcia, halloween, vendas, egipto antiguo</t>
         </is>
       </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>momia</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1796,6 +1982,11 @@
           <t>pastora, pastor de belen, biblico, nacimiento, pesebre, pase del nino</t>
         </is>
       </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>pastor-belen</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1831,6 +2022,11 @@
           <t>pirata, corsario, tesoro, tricornio, aventura, mar</t>
         </is>
       </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>pirata-clasico</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1866,6 +2062,11 @@
           <t>policia, oficial, uniforme, profesion, ley</t>
         </is>
       </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>policia</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -1901,6 +2102,11 @@
           <t>saragurena, saraguro, indigena, ecuador, folclorico, tradicional</t>
         </is>
       </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>saraguro</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1936,6 +2142,11 @@
           <t>vampira, dracula, halloween, capa, colmillos, gotico</t>
         </is>
       </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>vampiro-clasico</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -1971,6 +2182,11 @@
           <t>zombie, zombi, halloween, muerto viviente, terror</t>
         </is>
       </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>zombie</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2006,6 +2222,11 @@
           <t>abeja, insecto, animal, disfraz infantil, colmena</t>
         </is>
       </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>abeja</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2041,6 +2262,11 @@
           <t>arbol de navidad, navidad, pino navideno, disfraz infantil</t>
         </is>
       </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>arbol-navidad</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2076,6 +2302,11 @@
           <t>calabaza, jack o lantern, halloween, disfraz infantil</t>
         </is>
       </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>calabaza</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2111,6 +2342,11 @@
           <t>chola cuencana, chola, cuenca, folclorico, ecuador, disfraz infantil, pase del nino</t>
         </is>
       </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>chola-cuencana</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2146,6 +2382,11 @@
           <t>duende navideno, duende, navidad, elfo, disfraz infantil</t>
         </is>
       </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>duende-navidad</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2181,6 +2422,11 @@
           <t>mariposa, insecto, alas, animal, disfraz infantil</t>
         </is>
       </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>mariposa</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2216,6 +2462,11 @@
           <t>pastora, pastor de belen, biblico, nacimiento, pesebre, pase del nino, disfraz infantil</t>
         </is>
       </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>pastor-belen</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2251,6 +2502,11 @@
           <t>unicornio, fantasia, animal magico, disfraz infantil</t>
         </is>
       </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>unicornio</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2286,6 +2542,11 @@
           <t>angel, biblico, nacimiento, pesebre, pase del nino, alas, disfraz infantil</t>
         </is>
       </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>angel</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -2321,6 +2582,11 @@
           <t>conejo, orejas largas, animal, disfraz infantil, pascua</t>
         </is>
       </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>conejo</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2356,6 +2622,11 @@
           <t>duende travieso, duende, gnomo, bosque, disfraz infantil</t>
         </is>
       </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>duende-travieso</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2391,6 +2662,11 @@
           <t>estrella de navidad, estrella, navidad, disfraz infantil</t>
         </is>
       </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>estrella-navidad</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2426,6 +2702,11 @@
           <t>explorador, safari, selva, aventurero, disfraz infantil</t>
         </is>
       </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>explorador-selva</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2461,6 +2742,11 @@
           <t>leon, melena, animal, rey de la selva, disfraz infantil</t>
         </is>
       </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>leon</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -2496,6 +2782,11 @@
           <t>montubio, costa, ecuador, folclorico, tradicional, disfraz infantil</t>
         </is>
       </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>montubio</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -2529,6 +2820,11 @@
       <c r="G59" s="4" t="inlineStr">
         <is>
           <t>robot, mecanico, futurista, disfraz infantil</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>robot-ayudante</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2563,7 +2859,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>INSTRUCCIONES - CATÁLOGO DEMO CON 58 DISFRACES (IA)</t>
+          <t>INSTRUCCIONES - V6</t>
         </is>
       </c>
     </row>
@@ -2573,28 +2869,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. ESTRUCTURA DE CARPETAS</t>
+          <t>NUEVA COLUMNA: Grupo de Diseño</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Sube la carpeta 'disfraces' completa (con sus 4 subcarpetas: hombre, mujer, nina, nino)</t>
+          <t xml:space="preserve">   Si dos disfraces son 'la misma prenda' en distinto personaje (ej: vampiro/vampira,</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   dentro de images/ en tu repositorio, reemplazando la carpeta plana anterior.</t>
+          <t xml:space="preserve">   montubio hombre/niño, chola mujer/niña), ponles el MISMO valor en esta columna.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Resultado: images/disfraces/hombre/, images/disfraces/mujer/, images/disfraces/nina/, images/disfraces/nino/</t>
+          <t xml:space="preserve">   El sitio los agrupará automáticamente en una sola tarjeta con flechas para navegar.</t>
         </is>
       </c>
     </row>
@@ -2604,96 +2900,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2. NO SE NECESITA NINGÚN CAMBIO DE CÓDIGO</t>
+          <t xml:space="preserve">   Si un disfraz es único (sin variante en otro personaje), igual necesita un valor</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   La columna 'Nombre del Archivo' ya incluye la subcarpeta (ej: hombre/bombero.png)</t>
+          <t xml:space="preserve">   en esta columna (puede ser único, ej: 'bombero') - así queda listo para cuando</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   El GitHub Action arma la ruta automáticamente: images/disfraces/hombre/bombero.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>3. CATEGORÍAS NUEVAS (reemplazan a las 9 anteriores)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   halloween, navidad, religioso, tradicional, animados, animales, profesiones, epoca</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   IMPORTANTE: debes actualizar el &lt;select&gt; de categorías en index.html para que coincida</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   (quitar: carnaval, superheroes, princesas, infantiles / agregar: religioso, tradicional, animados)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>4. COLUMNA NUEVA: PALABRAS CLAVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Esta columna aún NO es usada por el buscador actual (filters.js).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Se necesita un pequeño cambio en filters.js para que incluya este campo en la búsqueda.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>EDADES: nino, adulto</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>GÉNEROS: hombre, mujer, nina, nino, unisex</t>
+          <t xml:space="preserve">   agregues una variante en el futuro.</t>
         </is>
       </c>
     </row>

</xml_diff>